<commit_message>
Adiciona lançamento: Maiora (13/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -532,6 +532,31 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Maiora</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>87</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: train bari-polignano (13/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -557,6 +557,31 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>train bari-polignano</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: bus J3 et J4 (13/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -582,6 +582,31 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>bus J3 et J4</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: dîner guide avec clients (13/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -607,6 +607,31 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>dîner guide avec clients (1 pizza+l'eau+couvert)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: maiora (14/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -632,6 +632,31 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>maiora</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: bus Alberobello Locorotondo (15/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -657,6 +657,31 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>bus Alberobello Locorotondo</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: maiora 72,78€ (14/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -682,6 +682,31 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>maiora</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>72.78</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: train Ostuni Lecce (17/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -707,6 +707,31 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>train Ostuni Lecce</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: mudo mosaïque Otranto (18/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -732,6 +732,31 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>mudo mosaïque Otranto</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: panificio (16/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -757,6 +757,31 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>panificio</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: alimentari (16/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -782,6 +782,31 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>alimentari</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: il delfino (17/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -807,6 +807,31 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>il delfino</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: bottega italiana (17/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -832,6 +832,31 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>bottega italiana</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: artigiana puglia (17/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -857,6 +857,31 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>artigiana puglia</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: Rapa ITI (18/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -882,6 +882,31 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Rapa ITI</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>252</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: train lecce Bari (18/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -907,6 +907,31 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>train lecce Bari</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>184.8</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: train bari-aeroport (18/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
+++ b/planilha/Séjour Pouilles du Sud 13-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -932,6 +932,31 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>train bari-aeroport</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>